<commit_message>
Money answers go one way; the Desk stops looping on short screens
G-01  Dex added a customer's Rs 11,50,000 to the Rs 1,68,000 yarn bill when
      asked what we owe suppliers. The side is now read from the question
      by code: supplier questions read supplier bills, customer questions
      sales invoices, and a question naming neither shows "Customers owe
      us" and "We owe suppliers" apart -- never one Outstanding.
F-01  The Finance "Ask AI" gets both lists on every tab (it had no bills on
      Revenue/Assets/Inventory) and ledger.ask 1.1 names which way each
      figure goes. Golden set: evals/cases/finance.py (replay + live pass).
A-42  The Desk's phone card gave its room back, fell short, asked again --
      in one commit, forever. Given back once per screen size now.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -14393,12 +14393,12 @@
       </c>
       <c r="H58" s="26" t="inlineStr">
         <is>
-          <t>Partly fixed</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="I58" s="26" t="inlineStr">
         <is>
-          <t>PARTLY FIXED 2026-10-08 (with F-04): the Finance AI context now carries payables_outstanding and payables_due (every unpaid purchase bill incl. those booked as stock). G-01 (Dex mixing receivables into "what we owe") still open.</t>
+          <t>FIXED 2026-10-09 (awaiting push): with F-04 the Finance AI context carries payables_outstanding / payables_due (bills booked as stock included); now /ledger/ask gets BOTH sides on every tab (it had no bill list on Revenue/Assets/Inventory), and ledger.ask 1.1 names which way each figure goes and forbids adding them. Golden set: evals/cases/finance.py (2 cases, pass replay AND live). Live on the scratch DB: "You owe Rs 1,68,000 to Sri Lakshmi Yarn Mills (SLY-4471, booked as inventory), due 5 Nov".</t>
         </is>
       </c>
     </row>
@@ -14714,10 +14714,14 @@
       </c>
       <c r="H65" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I65" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I65" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): routers/brain money_side() reads supplier vs customer from the question by code; supplier questions read purchase bills only (and an expenses plan becomes invoices), customer questions sales invoices only, and a question naming neither shows "Customers owe us" and "We owe suppliers" separately -- never one Outstanding. Rows say "Supplier bill (we owe)" / "Sales invoice (owed to us)". Live: Dex -&gt; "1 outstanding supplier bill totalling Rs 1,68,000 ... due 5 November 2026".</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="24" t="inlineStr">
@@ -16139,12 +16143,12 @@
       </c>
       <c r="H96" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="I96" s="26" t="inlineStr">
         <is>
-          <t>Found 2026-10-09 while checking C-13; split out as its own task (not part of this batch).</t>
+          <t>FIXED 2026-10-09 (awaiting push): Desk.js PhoneTabCard: tight is given back at most once per screen size (resize resets), and after it a shortfall must be seen afresh on new frames. Was: 9px untight / 45px tight, 45 &gt; 2x9, release, 9px, ask again in the same commit, forever. Checked 840x602, 360x640, 375x667, 390x844, 440x956 with 2 and 6 decisions, all three tabs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Approval only above a value; leave goes to who can approve it
B-03  A stage's approval gate takes an optional value: at or under it the
      card leaves without the sign-off; over it, or with no value, it waits
      and says why. Settings > Operations sets it, the card view explains
      it, and the sign-up interview can produce it (approval_rules 1.2,
      kind stage_signoff; golden case passes live).
D-04  With no manager and no sign-up rule, leave goes to a lead in the
      person's own team, then an HR team, then anyone who can approve
      leave, before the owner. Leave dates read "15-16 Oct".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -13020,12 +13020,12 @@
       </c>
       <c r="H27" s="26" t="inlineStr">
         <is>
-          <t>Partly fixed</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="I27" s="26" t="inlineStr">
         <is>
-          <t>PARTLY FIXED with B-01: value-based sign-off stage (approval_delegate) now exists and is editable in Settings &gt; Operations. Per-stage gate conditions beyond the sign-off stage still open.</t>
+          <t>FIXED 2026-10-09 (awaiting push): a stage approval gate takes an optional value ("only above Rs X"): Settings &gt; Operations &gt; a stage &gt; Approval to leave this stage &gt; only above. At or under it the card leaves without the sign-off; over it, or with no value, it waits ("awaiting owner approval (needed above Rs 5,00,000)"). The card view says "it is over Rs X" or "No sign-off needed". The sign-up interview can set it too (generators.approval_rules 1.2, kind stage_signoff; golden case passes live). Live: 3L card moved on when its tasks were done; 7L and no-value cards waited.</t>
         </is>
       </c>
     </row>
@@ -15031,10 +15031,14 @@
       </c>
       <c r="H72" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I72" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I72" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): leave approver chain: reporting manager &gt; per-team mapping &gt; team from sign-up &gt; NEW: a lead in the person's own team who can approve leave &gt; a member of an HR/people team who can (HR teams start with leave_approve) &gt; anyone else who can &gt; the owner. Dates: "15-16 Oct" / "30 Oct - 2 Nov" on the Leave page and in the leave messages. Live: a sales member's leave went to Kavitha in HR; the page read "15-16 Oct".</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Work already there: no twin tasks, proof before close, approve shows at once
C-14  A decision's task is compared with the open work already on its card
      (and, more strictly, anywhere). The review shows "Already on <card>:
      <task> - who - due" with Use that task / Add as new; approving uses
      the existing task (new person and date, decision linked) instead of
      adding a twin -- "1 existing task updated".
C-10  The Move-on box no longer closes a task that asks for proof without
      it: shown as "Needs proof" with Done off, carried on with the card.
C-15  After Approve the window draws the approved decision from the answer
      instead of the old "ready for you" copy until a re-read.
C-18  Routine set-up suggests a member of the team the routine is about,
      the owner only when that team has nobody yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -13912,10 +13912,14 @@
       </c>
       <c r="H47" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I47" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I47" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): the Move-on box no longer closes a task that asks for proof without proof: the server carries it on with the card (counted as needs_proof) and the box shows "Needs proof - attach it on the task to close it" with Done off; "Set all: Done" skips it. Live: carried to Quality Check.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
@@ -14088,10 +14092,14 @@
       </c>
       <c r="H51" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I51" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I51" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): services/voice.find_existing_work compares each proposed task with the open work already there -- on its card (the card's customer is implied, so "send the revised quotation to Northwind" matches "Send a preliminary quotation to the customer") and, more strictly, anywhere else. The review shows "Already on &lt;card&gt;: &lt;task&gt; - &lt;who&gt; - due &lt;date&gt;" with Use that task / Add as new; approving with Use updates that task's person and date, links the decision, and says "1 existing task updated" -- no twin. Live: quotation task moved to Fri 9 Oct, card still had two tasks.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="24" t="inlineStr">
@@ -14131,10 +14139,14 @@
       </c>
       <c r="H52" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I52" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I52" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): after Approve the window draws the approved decision from the answer itself (it waited for a re-read, seconds later, showing the old "ready for you" screen). "Approving..." shows while it works. Live: ~7 s on this laptop (cloud DB, ~220 ms a query), the window switched the moment it answered.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="24" t="inlineStr">
@@ -14260,10 +14272,14 @@
       </c>
       <c r="H55" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I55" s="26" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I55" s="26" t="inlineStr">
+        <is>
+          <t>FIXED 2026-10-09 (awaiting push): routine set-up suggests a member of the team the routine is about (its category, else its words, via shared/roles.resolve_role); the owner only when that team has nobody. The picker says "from the &lt;team&gt; team". Live: loom routines -&gt; Murugan (Loom Production).</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="24" t="inlineStr">

</xml_diff>